<commit_message>
updated real constants excels
</commit_message>
<xml_diff>
--- a/tests/ITER_2D_APEC/input_template.xlsx
+++ b/tests/ITER_2D_APEC/input_template.xlsx
@@ -1,29 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PlasmaArc\tests\ITER_2D_APEC\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D7694F5-838C-4539-B8AE-D1FFB3BE0D38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="4"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="element_types"/>
-    <sheet r:id="rId2" sheetId="2" name="cp"/>
-    <sheet r:id="rId3" sheetId="3" name="cpcyc"/>
-    <sheet r:id="rId4" sheetId="4" name="materials"/>
-    <sheet r:id="rId5" sheetId="5" name="real_constants"/>
-    <sheet r:id="rId6" sheetId="6" name="solver_settings"/>
-    <sheet r:id="rId7" sheetId="7" name="time_parameters"/>
-    <sheet r:id="rId8" sheetId="8" name="elem"/>
-    <sheet r:id="rId9" sheetId="9" name="node"/>
-    <sheet r:id="rId10" sheetId="10" name="transient_analysis"/>
+    <sheet name="element_types" sheetId="1" r:id="rId1"/>
+    <sheet name="cp" sheetId="2" r:id="rId2"/>
+    <sheet name="cpcyc" sheetId="3" r:id="rId3"/>
+    <sheet name="materials" sheetId="4" r:id="rId4"/>
+    <sheet name="real_constants" sheetId="5" r:id="rId5"/>
+    <sheet name="solver_settings" sheetId="6" r:id="rId6"/>
+    <sheet name="time_parameters" sheetId="7" r:id="rId7"/>
+    <sheet name="elem" sheetId="8" r:id="rId8"/>
+    <sheet name="node" sheetId="9" r:id="rId9"/>
+    <sheet name="transient_analysis" sheetId="10" r:id="rId10"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="110">
   <si>
     <t>time_step_number</t>
   </si>
@@ -196,21 +202,6 @@
     <t>ansys_real_constant</t>
   </si>
   <si>
-    <t>CARE</t>
-  </si>
-  <si>
-    <t>TURN</t>
-  </si>
-  <si>
-    <t>LENG</t>
-  </si>
-  <si>
-    <t>DIRZ</t>
-  </si>
-  <si>
-    <t>FILL</t>
-  </si>
-  <si>
     <t>SC</t>
   </si>
   <si>
@@ -359,12 +350,21 @@
   </si>
   <si>
     <t>PLANE233</t>
+  </si>
+  <si>
+    <t>THK</t>
+  </si>
+  <si>
+    <t>VC</t>
+  </si>
+  <si>
+    <t>CPSIGN</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.000000"/>
   </numFmts>
@@ -416,59 +416,51 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+  <cellXfs count="12">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -479,10 +471,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -520,71 +512,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -612,7 +604,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -635,11 +627,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -648,13 +640,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -664,7 +656,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -673,7 +665,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -682,7 +674,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -690,10 +682,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -758,51 +750,48 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="14" width="13.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="14.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="13.28515625" style="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="13.5703125" style="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="13.5703125" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="G1" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    </row>
+    <row r="2" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>21</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>111</v>
+      <c r="B2" t="s">
+        <v>106</v>
       </c>
       <c r="C2" s="1">
         <v>0</v>
@@ -820,12 +809,12 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row r="3" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>23</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>111</v>
+      <c r="B3" t="s">
+        <v>106</v>
       </c>
       <c r="C3" s="1">
         <v>3</v>
@@ -843,12 +832,12 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row r="4" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>24</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>111</v>
+      <c r="B4" t="s">
+        <v>106</v>
       </c>
       <c r="C4" s="1">
         <v>4</v>
@@ -866,12 +855,11 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="12"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
+    <row r="5" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
     </row>
@@ -881,24 +869,24 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="5" width="18.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="5" width="22.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="7" width="16.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="7" width="19.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="7" width="21.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="7" width="21.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="18.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -908,175 +896,175 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" s="2">
-        <v>0.0001</v>
+        <v>1E-4</v>
       </c>
       <c r="C2" s="1">
         <v>1</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" t="s">
         <v>9</v>
       </c>
       <c r="F2" s="2">
         <v>0.5</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" t="s">
         <v>9</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row r="3" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2</v>
       </c>
       <c r="B3" s="2">
-        <v>0.0002</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="C3" s="1">
         <v>4</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" t="s">
         <v>9</v>
       </c>
       <c r="F3" s="2">
         <v>0.5</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" t="s">
         <v>9</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row r="4" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
       <c r="B4" s="2">
-        <v>0.0003</v>
+        <v>2.9999999999999997E-4</v>
       </c>
       <c r="C4" s="1">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" t="s">
         <v>9</v>
       </c>
       <c r="F4" s="2">
         <v>0.5</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" t="s">
         <v>9</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row r="5" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
       <c r="B5" s="2">
-        <v>0.0004</v>
+        <v>4.0000000000000002E-4</v>
       </c>
       <c r="C5" s="1">
         <v>4</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" t="s">
         <v>9</v>
       </c>
       <c r="F5" s="2">
         <v>0.5</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row r="6" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
       <c r="B6" s="2">
-        <v>0.0005</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="C6" s="1">
         <v>4</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" t="s">
         <v>9</v>
       </c>
       <c r="F6" s="2">
         <v>0.5</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" t="s">
         <v>9</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="H6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row r="7" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
       <c r="B7" s="2">
-        <v>0.006</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="C7" s="1">
         <v>1</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" t="s">
         <v>9</v>
       </c>
       <c r="F7" s="2">
         <v>0.5</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="G7" t="s">
         <v>9</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="H7" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1086,57 +1074,42 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="13.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="5" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
-      <c r="A1" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row r="1" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="B1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D1" t="s">
+        <v>96</v>
+      </c>
+      <c r="E1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    </row>
+    <row r="3" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    </row>
+    <row r="4" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1144,68 +1117,57 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="9" width="14.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="7.147857142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="14.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="6" width="13.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="10" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="F1" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="G1" t="s">
         <v>94</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="H1" t="s">
         <v>95</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="I1" t="s">
         <v>96</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="J1" t="s">
         <v>97</v>
       </c>
-      <c r="F1" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    </row>
+    <row r="2" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
-      <c r="B2" s="3"/>
       <c r="C2" s="2"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1213,189 +1175,178 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:M4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="5" width="20.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="13" width="13.5703125" style="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="G1" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="H1" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="I1" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="J1" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="K1" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="L1" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="M1" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="I1" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="J1" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="K1" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="L1" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="M1" s="10" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    </row>
+    <row r="2" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>21</v>
       </c>
-      <c r="B2" s="10">
-        <v>1</v>
-      </c>
-      <c r="C2" s="10">
-        <v>1</v>
-      </c>
-      <c r="D2" s="10">
-        <v>1</v>
-      </c>
-      <c r="E2" s="10">
-        <v>0</v>
-      </c>
-      <c r="F2" s="10">
-        <v>0</v>
-      </c>
-      <c r="G2" s="10">
-        <v>0</v>
-      </c>
-      <c r="H2" s="10">
-        <v>0</v>
-      </c>
-      <c r="I2" s="10">
-        <v>0</v>
-      </c>
-      <c r="J2" s="10">
-        <v>0</v>
-      </c>
-      <c r="K2" s="10">
-        <v>0</v>
-      </c>
-      <c r="L2" s="10">
-        <v>0</v>
-      </c>
-      <c r="M2" s="10">
-        <v>0</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+      <c r="B2" s="8">
+        <v>1</v>
+      </c>
+      <c r="C2" s="8">
+        <v>1</v>
+      </c>
+      <c r="D2" s="8">
+        <v>1</v>
+      </c>
+      <c r="E2" s="8">
+        <v>0</v>
+      </c>
+      <c r="F2" s="8">
+        <v>0</v>
+      </c>
+      <c r="G2" s="8">
+        <v>0</v>
+      </c>
+      <c r="H2" s="8">
+        <v>0</v>
+      </c>
+      <c r="I2" s="8">
+        <v>0</v>
+      </c>
+      <c r="J2" s="8">
+        <v>0</v>
+      </c>
+      <c r="K2" s="8">
+        <v>0</v>
+      </c>
+      <c r="L2" s="8">
+        <v>0</v>
+      </c>
+      <c r="M2" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>23</v>
       </c>
-      <c r="B3" s="10">
-        <v>1</v>
-      </c>
-      <c r="C3" s="10">
-        <v>1</v>
-      </c>
-      <c r="D3" s="10">
-        <v>1</v>
-      </c>
-      <c r="E3" s="10">
-        <v>0</v>
-      </c>
-      <c r="F3" s="10">
-        <v>0</v>
-      </c>
-      <c r="G3" s="10">
-        <v>0</v>
-      </c>
-      <c r="H3" s="10">
-        <v>0</v>
-      </c>
-      <c r="I3" s="10">
-        <v>0</v>
-      </c>
-      <c r="J3" s="10">
-        <v>0</v>
-      </c>
-      <c r="K3" s="10">
-        <v>0</v>
-      </c>
-      <c r="L3" s="10">
-        <v>0</v>
-      </c>
-      <c r="M3" s="10">
-        <v>0</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+      <c r="B3" s="8">
+        <v>1</v>
+      </c>
+      <c r="C3" s="8">
+        <v>1</v>
+      </c>
+      <c r="D3" s="8">
+        <v>1</v>
+      </c>
+      <c r="E3" s="8">
+        <v>0</v>
+      </c>
+      <c r="F3" s="8">
+        <v>0</v>
+      </c>
+      <c r="G3" s="8">
+        <v>0</v>
+      </c>
+      <c r="H3" s="8">
+        <v>0</v>
+      </c>
+      <c r="I3" s="8">
+        <v>0</v>
+      </c>
+      <c r="J3" s="8">
+        <v>0</v>
+      </c>
+      <c r="K3" s="8">
+        <v>0</v>
+      </c>
+      <c r="L3" s="8">
+        <v>0</v>
+      </c>
+      <c r="M3" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>24</v>
       </c>
-      <c r="B4" s="10">
-        <v>1</v>
-      </c>
-      <c r="C4" s="10">
-        <v>1</v>
-      </c>
-      <c r="D4" s="10">
-        <v>1</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="F4" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="G4" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="H4" s="10">
-        <v>0</v>
-      </c>
-      <c r="I4" s="10">
-        <v>0</v>
-      </c>
-      <c r="J4" s="10">
-        <v>0</v>
-      </c>
-      <c r="K4" s="10">
-        <v>0</v>
-      </c>
-      <c r="L4" s="10">
-        <v>0</v>
-      </c>
-      <c r="M4" s="10">
+      <c r="B4" s="8">
+        <v>1</v>
+      </c>
+      <c r="C4" s="8">
+        <v>1</v>
+      </c>
+      <c r="D4" s="8">
+        <v>1</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="H4" s="8">
+        <v>0</v>
+      </c>
+      <c r="I4" s="8">
+        <v>0</v>
+      </c>
+      <c r="J4" s="8">
+        <v>0</v>
+      </c>
+      <c r="K4" s="8">
+        <v>0</v>
+      </c>
+      <c r="L4" s="8">
+        <v>0</v>
+      </c>
+      <c r="M4" s="8">
         <v>0</v>
       </c>
     </row>
@@ -1405,111 +1356,85 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:W3"/>
+  <dimension ref="A1:U3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="5" width="21.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="6.2907142857142855" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="5" width="6.2907142857142855" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="5" width="6.2907142857142855" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="5" width="6.2907142857142855" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="5" width="6.2907142857142855" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="5" width="6.2907142857142855" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="5" width="6.2907142857142855" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="5" width="6.2907142857142855" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="5" width="6.2907142857142855" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="5" width="6.2907142857142855" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="5" width="6.2907142857142855" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="5" width="6.2907142857142855" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="21.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="13" width="6.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="21" width="13.5703125" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="C1" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="D1" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="E1" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="F1" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="G1" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="H1" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="I1" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="J1" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="K1" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="L1" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="K1" s="12" t="s">
+      <c r="M1" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="L1" s="12" t="s">
+      <c r="N1" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="M1" s="12" t="s">
+      <c r="O1" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="N1" s="12" t="s">
+      <c r="P1" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="O1" s="12" t="s">
+      <c r="Q1" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="P1" s="12" t="s">
+      <c r="R1" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="Q1" s="12" t="s">
+      <c r="S1" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="R1" s="12" t="s">
+      <c r="T1" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="S1" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="T1" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="U1" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="V1" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="W1" s="12" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="13">
+      <c r="U1" s="10" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
       <c r="B2" s="1">
@@ -1572,14 +1497,8 @@
       <c r="U2" s="1">
         <v>0</v>
       </c>
-      <c r="V2" s="1">
-        <v>0</v>
-      </c>
-      <c r="W2" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    </row>
+    <row r="3" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1641,12 +1560,6 @@
         <v>0</v>
       </c>
       <c r="U3" s="1">
-        <v>0</v>
-      </c>
-      <c r="V3" s="1">
-        <v>0</v>
-      </c>
-      <c r="W3" s="1">
         <v>0</v>
       </c>
     </row>
@@ -1656,279 +1569,279 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="34.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="11" width="12.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="34" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" style="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="8" t="s">
         <v>21</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="8" t="s">
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="8" t="s">
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="10">
-        <v>0.000001</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="3" t="s">
+      <c r="B4" s="8">
+        <v>9.9999999999999995E-7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>27</v>
       </c>
       <c r="B5" s="1">
         <v>100</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="10">
-        <v>1e-10</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="3" t="s">
+      <c r="B6" s="8">
+        <v>1E-10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>29</v>
       </c>
       <c r="B7" s="1">
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="3" t="s">
+    <row r="8" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>30</v>
       </c>
       <c r="B8" s="1">
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
-      <c r="A9" s="3" t="s">
+    <row r="9" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="10">
-        <v>0.000001</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
-      <c r="A10" s="3" t="s">
+      <c r="B9" s="8">
+        <v>9.9999999999999995E-7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>32</v>
       </c>
       <c r="B10" s="1">
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
-      <c r="A11" s="3" t="s">
+    <row r="11" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>33</v>
       </c>
       <c r="B11" s="1">
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
-      <c r="A12" s="3" t="s">
+    <row r="12" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="10">
-        <v>0.000001</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
-      <c r="A13" s="3" t="s">
+      <c r="B12" s="8">
+        <v>9.9999999999999995E-7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>35</v>
       </c>
       <c r="B13" s="1">
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
-      <c r="A14" s="3" t="s">
+    <row r="14" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>36</v>
       </c>
       <c r="B14" s="1">
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
-      <c r="A15" s="3" t="s">
+    <row r="15" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>37</v>
       </c>
-      <c r="B15" s="10">
-        <v>0.000001</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
-      <c r="A16" s="3" t="s">
+      <c r="B15" s="8">
+        <v>9.9999999999999995E-7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>38</v>
       </c>
-      <c r="B16" s="10">
-        <v>0.000001</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
-      <c r="A17" s="3" t="s">
+      <c r="B16" s="8">
+        <v>9.9999999999999995E-7</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>39</v>
       </c>
       <c r="B17" s="1">
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
-      <c r="A18" s="3" t="s">
+    <row r="18" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>40</v>
       </c>
       <c r="B18" s="1">
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
-      <c r="A19" s="3" t="s">
+    <row r="19" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>41</v>
       </c>
       <c r="B19" s="1">
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
-      <c r="A20" s="3" t="s">
+    <row r="20" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>42</v>
       </c>
       <c r="B20" s="1">
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
-      <c r="A21" s="3" t="s">
+    <row r="21" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>43</v>
       </c>
       <c r="B21" s="1">
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
-      <c r="A22" s="3" t="s">
+    <row r="22" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>44</v>
       </c>
       <c r="B22" s="1">
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
-      <c r="A23" s="3" t="s">
+    <row r="23" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>45</v>
       </c>
       <c r="B23" s="1">
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
-      <c r="A24" s="3" t="s">
+    <row r="24" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>46</v>
       </c>
       <c r="B24" s="1">
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
-      <c r="A25" s="3" t="s">
+    <row r="25" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>47</v>
       </c>
       <c r="B25" s="1">
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
-      <c r="A26" s="3" t="s">
+    <row r="26" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>48</v>
       </c>
       <c r="B26" s="1">
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
-      <c r="A27" s="3" t="s">
+    <row r="27" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>49</v>
       </c>
       <c r="B27" s="1">
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
-      <c r="A28" s="3" t="s">
+    <row r="28" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>50</v>
       </c>
       <c r="B28" s="1">
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
-      <c r="A29" s="3" t="s">
+    <row r="29" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>51</v>
       </c>
       <c r="B29" s="1">
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
-      <c r="A30" s="3" t="s">
+    <row r="30" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>52</v>
       </c>
       <c r="B30" s="1">
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
-      <c r="A31" s="3" t="s">
+    <row r="31" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>53</v>
       </c>
       <c r="B31" s="1">
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
-      <c r="A32" s="3" t="s">
+    <row r="32" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>54</v>
       </c>
       <c r="B32" s="1">
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
-      <c r="A33" s="3" t="s">
+    <row r="33" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>55</v>
       </c>
-      <c r="B33" s="10">
-        <v>0.000001</v>
+      <c r="B33" s="8">
+        <v>9.9999999999999995E-7</v>
       </c>
     </row>
   </sheetData>
@@ -1937,75 +1850,75 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="23.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="11.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="10">
-        <v>0.0001</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="3" t="s">
+    <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="8">
+        <v>1E-4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="1">
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="1">
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="1">
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>5</v>
       </c>
       <c r="B7" s="1">
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="3" t="s">
+    <row r="8" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>6</v>
       </c>
       <c r="B8" s="1">
@@ -2018,78 +1931,70 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="9" width="15.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="6.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="9" width="11.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="15.42578125" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5703125" style="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="6" t="s">
         <v>19</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="8"/>
-      <c r="B2" s="3"/>
+    <row r="2" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="6"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="8"/>
-      <c r="B3" s="3"/>
+    <row r="3" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="8"/>
-      <c r="B4" s="3"/>
+    <row r="4" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="6"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="8"/>
-      <c r="B5" s="3"/>
+    <row r="5" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="8"/>
-      <c r="B6" s="3"/>
+    <row r="6" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="6"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="8"/>
-      <c r="B7" s="3"/>
+    <row r="7" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="6"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="8"/>
-      <c r="B8" s="3"/>
+    <row r="8" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="6"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
-      <c r="A9" s="8"/>
-      <c r="B9" s="3"/>
+    <row r="9" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="6"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
     </row>
@@ -2099,108 +2004,95 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="9" width="16.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="17.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="9" width="12.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="16.42578125" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5703125" style="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="6" t="s">
         <v>19</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
+    <row r="2" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
-      <c r="B2" s="3"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
+    <row r="3" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
-      <c r="B3" s="3"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
+    <row r="4" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
-      <c r="B4" s="3"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
+    <row r="5" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
-      <c r="B5" s="3"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
+    <row r="6" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
-      <c r="B6" s="3"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
+    <row r="7" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
-      <c r="B7" s="3"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
+    <row r="8" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
-      <c r="B8" s="3"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
+    <row r="9" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
-      <c r="B9" s="3"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
+    <row r="10" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
-      <c r="B10" s="3"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
+    <row r="11" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
-      <c r="B11" s="3"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
+    <row r="12" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
-      <c r="B12" s="3"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
+    <row r="13" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
-      <c r="B13" s="3"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
+    <row r="14" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
-      <c r="B14" s="3"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
     </row>

</xml_diff>

<commit_message>
fixed many APEC issues
</commit_message>
<xml_diff>
--- a/tests/ITER_2D_APEC/input_template.xlsx
+++ b/tests/ITER_2D_APEC/input_template.xlsx
@@ -1,30 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PlasmaArc\tests\ITER_2D_APEC\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6B2D791-438D-47A8-9F8D-F9CE8639AC63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="4"/>
   </bookViews>
   <sheets>
-    <sheet name="element_types" sheetId="1" r:id="rId1"/>
-    <sheet name="cp" sheetId="2" r:id="rId2"/>
-    <sheet name="cpcyc" sheetId="3" r:id="rId3"/>
-    <sheet name="materials" sheetId="4" r:id="rId4"/>
-    <sheet name="real_constants" sheetId="5" r:id="rId5"/>
-    <sheet name="solver_settings" sheetId="6" r:id="rId6"/>
-    <sheet name="time_parameters" sheetId="7" r:id="rId7"/>
-    <sheet name="elem" sheetId="8" r:id="rId8"/>
-    <sheet name="node" sheetId="9" r:id="rId9"/>
-    <sheet name="transient_analysis" sheetId="10" r:id="rId10"/>
+    <sheet r:id="rId1" sheetId="1" name="element_types"/>
+    <sheet r:id="rId2" sheetId="2" name="cp"/>
+    <sheet r:id="rId3" sheetId="3" name="cpcyc"/>
+    <sheet r:id="rId4" sheetId="4" name="materials"/>
+    <sheet r:id="rId5" sheetId="5" name="real_constants"/>
+    <sheet r:id="rId6" sheetId="6" name="solver_settings"/>
+    <sheet r:id="rId7" sheetId="7" name="time_parameters"/>
+    <sheet r:id="rId8" sheetId="8" name="elem"/>
+    <sheet r:id="rId9" sheetId="9" name="node"/>
+    <sheet r:id="rId10" sheetId="10" name="transient_analysis"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -361,7 +355,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.000000"/>
   </numFmts>
@@ -413,47 +407,50 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="12">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle xfId="0" builtinId="0" name="Normal"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -464,10 +461,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -505,71 +502,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Times New Roman" script="Arab"/>
+        <a:font typeface="Times New Roman" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="MoolBoran" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Times New Roman" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Arial" script="Arab"/>
+        <a:font typeface="Arial" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="DaunPenh" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Arial" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -597,7 +594,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -620,11 +617,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -633,13 +630,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -649,7 +646,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -658,7 +655,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -667,7 +664,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -675,10 +672,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
+              <a:rot rev="0" lon="0" lat="0"/>
             </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
+            <a:lightRig dir="t" rig="threePt">
+              <a:rot rev="1200000" lon="0" lat="0"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -743,23 +740,27 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="7" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="4" width="13.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="14.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>102</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -778,11 +779,11 @@
         <v>107</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1">
         <v>21</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>108</v>
       </c>
       <c r="C2" s="1">
@@ -801,11 +802,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="1">
         <v>23</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="3" t="s">
         <v>108</v>
       </c>
       <c r="C3" s="1">
@@ -824,11 +825,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1">
         <v>24</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="3" t="s">
         <v>108</v>
       </c>
       <c r="C4" s="1">
@@ -847,8 +848,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="1"/>
+      <c r="B5" s="3"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
@@ -861,24 +863,24 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="4" width="18.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="4" width="22.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="6" width="16.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="6" width="19.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="6" width="21.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="6" width="21.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -888,175 +890,175 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" s="2">
-        <v>1E-4</v>
+        <v>0.0001</v>
       </c>
       <c r="C2" s="1">
         <v>1</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F2" s="2">
         <v>0.5</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="1">
         <v>2</v>
       </c>
       <c r="B3" s="2">
-        <v>2.0000000000000001E-4</v>
+        <v>0.0002</v>
       </c>
       <c r="C3" s="1">
         <v>4</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F3" s="2">
         <v>0.5</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1">
         <v>3</v>
       </c>
       <c r="B4" s="2">
-        <v>2.9999999999999997E-4</v>
+        <v>0.0003</v>
       </c>
       <c r="C4" s="1">
         <v>4</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F4" s="2">
         <v>0.5</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="1">
         <v>4</v>
       </c>
       <c r="B5" s="2">
-        <v>4.0000000000000002E-4</v>
+        <v>0.0004</v>
       </c>
       <c r="C5" s="1">
         <v>4</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F5" s="2">
         <v>0.5</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H5" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="1">
         <v>5</v>
       </c>
       <c r="B6" s="2">
-        <v>5.0000000000000001E-4</v>
+        <v>0.0005</v>
       </c>
       <c r="C6" s="1">
         <v>4</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F6" s="2">
         <v>0.5</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H6" t="s">
+      <c r="H6" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="1">
         <v>6</v>
       </c>
       <c r="B7" s="2">
-        <v>6.0000000000000001E-3</v>
+        <v>0.006</v>
       </c>
       <c r="C7" s="1">
         <v>1</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F7" s="2">
         <v>0.5</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H7" s="3" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1066,42 +1068,57 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="5" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+      <c r="A1" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1"/>
-    </row>
-    <row r="3" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="1"/>
-    </row>
-    <row r="4" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1109,57 +1126,68 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.28515625" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="6" width="13.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="10" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="8" width="14.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="7.147857142857143" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+      <c r="A1" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1"/>
+      <c r="B2" s="3"/>
       <c r="C2" s="2"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1167,178 +1195,189 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:M4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="13" width="13.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="4" width="20.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="I1" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="J1" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="K1" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="L1" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="M1" s="7" t="s">
+      <c r="M1" s="9" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1">
         <v>21</v>
       </c>
-      <c r="B2" s="7">
-        <v>1</v>
-      </c>
-      <c r="C2" s="7">
-        <v>1</v>
-      </c>
-      <c r="D2" s="7">
-        <v>1</v>
-      </c>
-      <c r="E2" s="7">
-        <v>0</v>
-      </c>
-      <c r="F2" s="7">
-        <v>0</v>
-      </c>
-      <c r="G2" s="7">
-        <v>0</v>
-      </c>
-      <c r="H2" s="7">
-        <v>0</v>
-      </c>
-      <c r="I2" s="7">
-        <v>0</v>
-      </c>
-      <c r="J2" s="7">
-        <v>0</v>
-      </c>
-      <c r="K2" s="7">
-        <v>0</v>
-      </c>
-      <c r="L2" s="7">
-        <v>0</v>
-      </c>
-      <c r="M2" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="9">
+        <v>1</v>
+      </c>
+      <c r="C2" s="9">
+        <v>1</v>
+      </c>
+      <c r="D2" s="9">
+        <v>1</v>
+      </c>
+      <c r="E2" s="9">
+        <v>0</v>
+      </c>
+      <c r="F2" s="9">
+        <v>0</v>
+      </c>
+      <c r="G2" s="9">
+        <v>0</v>
+      </c>
+      <c r="H2" s="9">
+        <v>0</v>
+      </c>
+      <c r="I2" s="9">
+        <v>0</v>
+      </c>
+      <c r="J2" s="9">
+        <v>0</v>
+      </c>
+      <c r="K2" s="9">
+        <v>0</v>
+      </c>
+      <c r="L2" s="9">
+        <v>0</v>
+      </c>
+      <c r="M2" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="1">
         <v>23</v>
       </c>
-      <c r="B3" s="7">
-        <v>1</v>
-      </c>
-      <c r="C3" s="7">
-        <v>1</v>
-      </c>
-      <c r="D3" s="7">
-        <v>1</v>
-      </c>
-      <c r="E3" s="7">
-        <v>0</v>
-      </c>
-      <c r="F3" s="7">
-        <v>0</v>
-      </c>
-      <c r="G3" s="7">
-        <v>0</v>
-      </c>
-      <c r="H3" s="7">
-        <v>0</v>
-      </c>
-      <c r="I3" s="7">
-        <v>0</v>
-      </c>
-      <c r="J3" s="7">
-        <v>0</v>
-      </c>
-      <c r="K3" s="7">
-        <v>0</v>
-      </c>
-      <c r="L3" s="7">
-        <v>0</v>
-      </c>
-      <c r="M3" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="9">
+        <v>1</v>
+      </c>
+      <c r="C3" s="9">
+        <v>1</v>
+      </c>
+      <c r="D3" s="9">
+        <v>1</v>
+      </c>
+      <c r="E3" s="9">
+        <v>0</v>
+      </c>
+      <c r="F3" s="9">
+        <v>0</v>
+      </c>
+      <c r="G3" s="9">
+        <v>0</v>
+      </c>
+      <c r="H3" s="9">
+        <v>0</v>
+      </c>
+      <c r="I3" s="9">
+        <v>0</v>
+      </c>
+      <c r="J3" s="9">
+        <v>0</v>
+      </c>
+      <c r="K3" s="9">
+        <v>0</v>
+      </c>
+      <c r="L3" s="9">
+        <v>0</v>
+      </c>
+      <c r="M3" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1">
         <v>24</v>
       </c>
-      <c r="B4" s="7">
-        <v>1</v>
-      </c>
-      <c r="C4" s="7">
-        <v>1</v>
-      </c>
-      <c r="D4" s="7">
-        <v>1</v>
-      </c>
-      <c r="E4" s="7">
-        <v>7.9999999999999996E-6</v>
-      </c>
-      <c r="F4" s="7">
-        <v>7.9999999999999996E-6</v>
-      </c>
-      <c r="G4" s="7">
-        <v>7.9999999999999996E-6</v>
-      </c>
-      <c r="H4" s="7">
-        <v>0</v>
-      </c>
-      <c r="I4" s="7">
-        <v>0</v>
-      </c>
-      <c r="J4" s="7">
-        <v>0</v>
-      </c>
-      <c r="K4" s="7">
-        <v>0</v>
-      </c>
-      <c r="L4" s="7">
-        <v>0</v>
-      </c>
-      <c r="M4" s="7">
+      <c r="B4" s="9">
+        <v>1</v>
+      </c>
+      <c r="C4" s="9">
+        <v>1</v>
+      </c>
+      <c r="D4" s="9">
+        <v>1</v>
+      </c>
+      <c r="E4" s="9">
+        <v>0.000008</v>
+      </c>
+      <c r="F4" s="9">
+        <v>0.000008</v>
+      </c>
+      <c r="G4" s="9">
+        <v>0.000008</v>
+      </c>
+      <c r="H4" s="9">
+        <v>0</v>
+      </c>
+      <c r="I4" s="9">
+        <v>0</v>
+      </c>
+      <c r="J4" s="9">
+        <v>0</v>
+      </c>
+      <c r="K4" s="9">
+        <v>0</v>
+      </c>
+      <c r="L4" s="9">
+        <v>0</v>
+      </c>
+      <c r="M4" s="9">
         <v>0</v>
       </c>
     </row>
@@ -1348,28 +1387,44 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:U9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.5703125" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="13" width="6.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="14" max="21" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="4" width="21.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="4" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="10" width="9.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="4" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="4" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="4" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="4" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="4" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="4" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="4" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="4" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="4" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="4" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>56</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="9" t="s">
         <v>58</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -1427,15 +1482,15 @@
         <v>76</v>
       </c>
     </row>
-    <row r="2" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="9">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
+      <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" s="1">
         <v>0</v>
       </c>
-      <c r="C2" s="7">
-        <v>0.94375189999999998</v>
+      <c r="C2" s="9">
+        <v>0.9437519</v>
       </c>
       <c r="D2" s="1">
         <v>0</v>
@@ -1492,15 +1547,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="3">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
+      <c r="A3" s="11">
         <v>2</v>
       </c>
       <c r="B3" s="1">
         <v>0</v>
       </c>
-      <c r="C3" s="7">
-        <v>0.41453946000000003</v>
+      <c r="C3" s="9">
+        <v>0.41453946</v>
       </c>
       <c r="D3" s="1">
         <v>0</v>
@@ -1554,18 +1609,18 @@
         <v>0</v>
       </c>
       <c r="U3" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
+      <c r="A4" s="11">
         <v>3</v>
       </c>
       <c r="B4" s="1">
         <v>0</v>
       </c>
-      <c r="C4" s="7">
-        <v>0.66413093999999995</v>
+      <c r="C4" s="9">
+        <v>0.66413094</v>
       </c>
       <c r="D4" s="1">
         <v>0</v>
@@ -1619,18 +1674,18 @@
         <v>0</v>
       </c>
       <c r="U4" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
+      <c r="A5" s="11">
         <v>4</v>
       </c>
       <c r="B5" s="1">
         <v>0</v>
       </c>
-      <c r="C5" s="7">
-        <v>0.60871516000000003</v>
+      <c r="C5" s="9">
+        <v>0.60871516</v>
       </c>
       <c r="D5" s="1">
         <v>0</v>
@@ -1684,17 +1739,17 @@
         <v>0</v>
       </c>
       <c r="U5" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
+      <c r="A6" s="11">
         <v>5</v>
       </c>
       <c r="B6" s="1">
         <v>0</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="9">
         <v>0.7749625</v>
       </c>
       <c r="D6" s="1">
@@ -1749,17 +1804,17 @@
         <v>0</v>
       </c>
       <c r="U6" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="3">
+        <v>-1</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
+      <c r="A7" s="11">
         <v>6</v>
       </c>
       <c r="B7" s="1">
         <v>0</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="9">
         <v>1.7265925</v>
       </c>
       <c r="D7" s="1">
@@ -1817,14 +1872,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="3">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
+      <c r="A8" s="11">
         <v>10</v>
       </c>
       <c r="B8" s="1">
         <v>0</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="9">
         <v>28.6027095</v>
       </c>
       <c r="D8" s="1">
@@ -1882,14 +1937,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="1">
         <v>20</v>
       </c>
       <c r="B9" s="1">
         <v>0</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C9" s="9">
         <v>0</v>
       </c>
       <c r="D9" s="1">
@@ -1953,279 +2008,279 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="6" width="34.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="10" width="12.147857142857141" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+      <c r="A1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="9" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+      <c r="A2" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="9" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+      <c r="A3" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+      <c r="A4" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="7">
-        <v>9.9999999999999995E-7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B4" s="9">
+        <v>0.000001</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+      <c r="A5" s="3" t="s">
         <v>27</v>
       </c>
       <c r="B5" s="1">
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+      <c r="A6" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="7">
-        <v>1E-10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="B6" s="9">
+        <v>1e-10</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+      <c r="A7" s="3" t="s">
         <v>29</v>
       </c>
       <c r="B7" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+      <c r="A8" s="3" t="s">
         <v>30</v>
       </c>
       <c r="B8" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+      <c r="A9" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="7">
-        <v>9.9999999999999995E-7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="B9" s="9">
+        <v>0.000001</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+      <c r="A10" s="3" t="s">
         <v>32</v>
       </c>
       <c r="B10" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+      <c r="A11" s="3" t="s">
         <v>33</v>
       </c>
       <c r="B11" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+      <c r="A12" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="7">
-        <v>9.9999999999999995E-7</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="B12" s="9">
+        <v>0.000001</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+      <c r="A13" s="3" t="s">
         <v>35</v>
       </c>
       <c r="B13" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+      <c r="A14" s="3" t="s">
         <v>36</v>
       </c>
       <c r="B14" s="1">
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+      <c r="A15" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B15" s="7">
-        <v>9.9999999999999995E-7</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="B15" s="9">
+        <v>0.000001</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+      <c r="A16" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B16" s="7">
-        <v>9.9999999999999995E-7</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="B16" s="9">
+        <v>0.000001</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+      <c r="A17" s="3" t="s">
         <v>39</v>
       </c>
       <c r="B17" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
+      <c r="A18" s="3" t="s">
         <v>40</v>
       </c>
       <c r="B18" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
+      <c r="A19" s="3" t="s">
         <v>41</v>
       </c>
       <c r="B19" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
+      <c r="A20" s="3" t="s">
         <v>42</v>
       </c>
       <c r="B20" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
+      <c r="A21" s="3" t="s">
         <v>43</v>
       </c>
       <c r="B21" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
+      <c r="A22" s="3" t="s">
         <v>44</v>
       </c>
       <c r="B22" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
+      <c r="A23" s="3" t="s">
         <v>45</v>
       </c>
       <c r="B23" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
+      <c r="A24" s="3" t="s">
         <v>46</v>
       </c>
       <c r="B24" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
+      <c r="A25" s="3" t="s">
         <v>47</v>
       </c>
       <c r="B25" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
+      <c r="A26" s="3" t="s">
         <v>48</v>
       </c>
       <c r="B26" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
+      <c r="A27" s="3" t="s">
         <v>49</v>
       </c>
       <c r="B27" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
+      <c r="A28" s="3" t="s">
         <v>50</v>
       </c>
       <c r="B28" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
+      <c r="A29" s="3" t="s">
         <v>51</v>
       </c>
       <c r="B29" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
+      <c r="A30" s="3" t="s">
         <v>52</v>
       </c>
       <c r="B30" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
+      <c r="A31" s="3" t="s">
         <v>53</v>
       </c>
       <c r="B31" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
+      <c r="A32" s="3" t="s">
         <v>54</v>
       </c>
       <c r="B32" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
+      <c r="A33" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B33" s="7">
-        <v>9.9999999999999995E-7</v>
+      <c r="B33" s="9">
+        <v>0.000001</v>
       </c>
     </row>
   </sheetData>
@@ -2234,75 +2289,75 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="6" width="23.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="4" width="11.290714285714287" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+      <c r="A1" s="3" t="s">
         <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="7">
-        <v>1E-4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+      <c r="A3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="9">
+        <v>0.0001</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+      <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+      <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B7" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+      <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B8" s="1">
@@ -2315,70 +2370,78 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.42578125" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.28515625" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="8" width="15.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="6.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="8" width="11.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+      <c r="A1" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="5"/>
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+      <c r="A2" s="7"/>
+      <c r="B2" s="3"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
     </row>
-    <row r="3" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="5"/>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+      <c r="A3" s="7"/>
+      <c r="B3" s="3"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
     </row>
-    <row r="4" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="5"/>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+      <c r="A4" s="7"/>
+      <c r="B4" s="3"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="5"/>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+      <c r="A5" s="7"/>
+      <c r="B5" s="3"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
     </row>
-    <row r="6" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="5"/>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+      <c r="A6" s="7"/>
+      <c r="B6" s="3"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
     </row>
-    <row r="7" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="5"/>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+      <c r="A7" s="7"/>
+      <c r="B7" s="3"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
     </row>
-    <row r="8" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="5"/>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+      <c r="A8" s="7"/>
+      <c r="B8" s="3"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
     </row>
-    <row r="9" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="5"/>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+      <c r="A9" s="7"/>
+      <c r="B9" s="3"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
     </row>
@@ -2388,95 +2451,108 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="8" width="16.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="17.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="8" width="12.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
+      <c r="A1" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="1"/>
+      <c r="B2" s="3"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
     </row>
-    <row r="3" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="1"/>
+      <c r="B3" s="3"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
     </row>
-    <row r="4" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="1"/>
+      <c r="B4" s="3"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="1"/>
+      <c r="B5" s="3"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
     </row>
-    <row r="6" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="1"/>
+      <c r="B6" s="3"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
     </row>
-    <row r="7" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="1"/>
+      <c r="B7" s="3"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
     </row>
-    <row r="8" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="1"/>
+      <c r="B8" s="3"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
     </row>
-    <row r="9" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="1"/>
+      <c r="B9" s="3"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
     </row>
-    <row r="10" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="1"/>
+      <c r="B10" s="3"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
     </row>
-    <row r="11" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="1"/>
+      <c r="B11" s="3"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
     </row>
-    <row r="12" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="1"/>
+      <c r="B12" s="3"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
     </row>
-    <row r="13" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="1"/>
+      <c r="B13" s="3"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
     </row>
-    <row r="14" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="1"/>
+      <c r="B14" s="3"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
     </row>

</xml_diff>

<commit_message>
converging 2D eddy currents coils
</commit_message>
<xml_diff>
--- a/tests/ITER_2D_APEC/input_template.xlsx
+++ b/tests/ITER_2D_APEC/input_template.xlsx
@@ -4,11 +4,11 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="3"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="element_types"/>
-    <sheet r:id="rId2" sheetId="2" name="cp"/>
+    <sheet r:id="rId2" sheetId="2" name="dof_couplings"/>
     <sheet r:id="rId3" sheetId="3" name="cpcyc"/>
     <sheet r:id="rId4" sheetId="4" name="materials"/>
     <sheet r:id="rId5" sheetId="5" name="real_constants"/>
@@ -410,7 +410,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -443,9 +443,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -1223,7 +1220,7 @@
     <col min="13" max="13" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>78</v>
       </c>
@@ -1264,7 +1261,7 @@
         <v>90</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="1">
         <v>21</v>
       </c>
@@ -1305,7 +1302,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="1">
         <v>23</v>
       </c>
@@ -1346,7 +1343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="1">
         <v>24</v>
       </c>
@@ -1485,10 +1482,10 @@
       <c r="T1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="U1" s="11" t="s">
+      <c r="U1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="V1" s="12" t="s">
+      <c r="V1" s="11" t="s">
         <v>77</v>
       </c>
     </row>
@@ -1556,7 +1553,7 @@
       <c r="U2" s="1">
         <v>0</v>
       </c>
-      <c r="V2" s="11">
+      <c r="V2" s="1">
         <v>5732500</v>
       </c>
     </row>
@@ -1624,7 +1621,7 @@
       <c r="U3" s="1">
         <v>1</v>
       </c>
-      <c r="V3" s="11">
+      <c r="V3" s="1">
         <v>-2883400</v>
       </c>
     </row>
@@ -1692,7 +1689,7 @@
       <c r="U4" s="1">
         <v>1</v>
       </c>
-      <c r="V4" s="11">
+      <c r="V4" s="1">
         <v>-5808400</v>
       </c>
     </row>
@@ -1760,7 +1757,7 @@
       <c r="U5" s="1">
         <v>1</v>
       </c>
-      <c r="V5" s="11">
+      <c r="V5" s="1">
         <v>-4776200</v>
       </c>
     </row>
@@ -1828,7 +1825,7 @@
       <c r="U6" s="1">
         <v>-1</v>
       </c>
-      <c r="V6" s="11">
+      <c r="V6" s="1">
         <v>-7813300</v>
       </c>
     </row>
@@ -1896,7 +1893,7 @@
       <c r="U7" s="1">
         <v>0</v>
       </c>
-      <c r="V7" s="11">
+      <c r="V7" s="1">
         <v>16941000</v>
       </c>
     </row>
@@ -1964,7 +1961,7 @@
       <c r="U8" s="1">
         <v>0</v>
       </c>
-      <c r="V8" s="11">
+      <c r="V8" s="1">
         <v>0</v>
       </c>
     </row>
@@ -2032,7 +2029,7 @@
       <c r="U9" s="1">
         <v>0</v>
       </c>
-      <c r="V9" s="11">
+      <c r="V9" s="1">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
evolution faster convergence and simplified input logic
</commit_message>
<xml_diff>
--- a/tests/ITER_2D_APEC/input_template.xlsx
+++ b/tests/ITER_2D_APEC/input_template.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="element_types"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="112">
   <si>
     <t>time_step_number</t>
   </si>
@@ -254,9 +254,6 @@
   </si>
   <si>
     <t>CPSIGN</t>
-  </si>
-  <si>
-    <t>CURR</t>
   </si>
   <si>
     <t>ansys_material_type</t>
@@ -761,25 +758,25 @@
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>111</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
@@ -787,7 +784,7 @@
         <v>21</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C2" s="1">
         <v>0</v>
@@ -810,7 +807,7 @@
         <v>23</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C3" s="1">
         <v>3</v>
@@ -833,7 +830,7 @@
         <v>24</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C4" s="1">
         <v>4</v>
@@ -856,7 +853,7 @@
         <v>25</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C5" s="1">
         <v>8</v>
@@ -1098,10 +1095,10 @@
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>101</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>102</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
@@ -1109,7 +1106,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
@@ -1117,7 +1114,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
@@ -1125,7 +1122,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
@@ -1133,7 +1130,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
@@ -1141,7 +1138,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
@@ -1149,7 +1146,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
@@ -1157,7 +1154,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
@@ -1165,7 +1162,7 @@
         <v>4</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
@@ -1173,7 +1170,7 @@
         <v>5</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
@@ -1181,7 +1178,7 @@
         <v>5</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
@@ -1189,7 +1186,7 @@
         <v>6</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
@@ -1197,7 +1194,7 @@
         <v>6</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
@@ -1205,7 +1202,7 @@
         <v>11</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
@@ -1213,7 +1210,7 @@
         <v>11</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
@@ -1221,7 +1218,7 @@
         <v>12</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
@@ -1229,7 +1226,7 @@
         <v>12</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
@@ -1237,7 +1234,7 @@
         <v>13</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
@@ -1245,7 +1242,7 @@
         <v>13</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
@@ -1253,7 +1250,7 @@
         <v>14</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
@@ -1261,7 +1258,7 @@
         <v>14</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
@@ -1269,7 +1266,7 @@
         <v>15</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
@@ -1277,7 +1274,7 @@
         <v>15</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
@@ -1285,7 +1282,7 @@
         <v>16</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
@@ -1293,7 +1290,7 @@
         <v>16</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -1323,34 +1320,34 @@
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="D1" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="E1" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="F1" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="G1" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>99</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>100</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
@@ -1395,43 +1392,43 @@
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="C1" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="D1" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="E1" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="F1" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="G1" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="H1" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="I1" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="J1" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="K1" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="L1" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="M1" s="9" t="s">
         <v>89</v>
-      </c>
-      <c r="M1" s="9" t="s">
-        <v>90</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
@@ -1608,7 +1605,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:V15"/>
+  <dimension ref="A1:U15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="4" width="21.14785714285714" customWidth="1" bestFit="1"/>
@@ -1632,7 +1629,6 @@
     <col min="19" max="19" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="20" max="20" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="21" max="21" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
@@ -1699,9 +1695,6 @@
       <c r="U1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="V1" s="1" t="s">
-        <v>77</v>
-      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="1">
@@ -1766,9 +1759,6 @@
       </c>
       <c r="U2" s="1">
         <v>0</v>
-      </c>
-      <c r="V2" s="1">
-        <v>5732500</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
@@ -1835,9 +1825,6 @@
       <c r="U3" s="1">
         <v>1</v>
       </c>
-      <c r="V3" s="1">
-        <v>-2883400</v>
-      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="1">
@@ -1903,9 +1890,6 @@
       <c r="U4" s="1">
         <v>1</v>
       </c>
-      <c r="V4" s="1">
-        <v>-5808400</v>
-      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="1">
@@ -1971,9 +1955,6 @@
       <c r="U5" s="1">
         <v>1</v>
       </c>
-      <c r="V5" s="1">
-        <v>-4776200</v>
-      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="1">
@@ -2039,9 +2020,6 @@
       <c r="U6" s="1">
         <v>-1</v>
       </c>
-      <c r="V6" s="1">
-        <v>-7813300</v>
-      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="1">
@@ -2107,9 +2085,6 @@
       <c r="U7" s="1">
         <v>0</v>
       </c>
-      <c r="V7" s="1">
-        <v>16941000</v>
-      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="1">
@@ -2175,9 +2150,6 @@
       <c r="U8" s="1">
         <v>0</v>
       </c>
-      <c r="V8" s="1">
-        <v>0</v>
-      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="1">
@@ -2243,9 +2215,6 @@
       <c r="U9" s="1">
         <v>0</v>
       </c>
-      <c r="V9" s="2">
-        <v>-4820400</v>
-      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="1">
@@ -2311,9 +2280,6 @@
       <c r="U10" s="1">
         <v>0</v>
       </c>
-      <c r="V10" s="1">
-        <v>-4048000</v>
-      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="1">
@@ -2379,9 +2345,6 @@
       <c r="U11" s="1">
         <v>0</v>
       </c>
-      <c r="V11" s="1">
-        <v>-20804000</v>
-      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="1">
@@ -2447,9 +2410,6 @@
       <c r="U12" s="1">
         <v>0</v>
       </c>
-      <c r="V12" s="1">
-        <v>-20804000</v>
-      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="1">
@@ -2515,9 +2475,6 @@
       <c r="U13" s="1">
         <v>0</v>
       </c>
-      <c r="V13" s="1">
-        <v>-10297000</v>
-      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="1">
@@ -2583,9 +2540,6 @@
       <c r="U14" s="1">
         <v>0</v>
       </c>
-      <c r="V14" s="1">
-        <v>5301200</v>
-      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
       <c r="A15" s="1">
@@ -2649,9 +2603,6 @@
         <v>0</v>
       </c>
       <c r="U15" s="1">
-        <v>0</v>
-      </c>
-      <c r="V15" s="1">
         <v>0</v>
       </c>
     </row>

</xml_diff>